<commit_message>
Aded the xlsx file of master data
</commit_message>
<xml_diff>
--- a/public/Master_Data_Upload_template.xlsx
+++ b/public/Master_Data_Upload_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10913"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lavanya\Desktop\Mold-TEK\Moldtek-UI\public\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABB32C06-02A2-4AE5-A0DD-0AB46C53D435}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{00218388-4E40-9E4E-92BC-E77B8EF3164B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8860" yWindow="3080" windowWidth="20740" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DropdownValues" sheetId="2" state="hidden" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="88">
   <si>
     <t>Type of Label</t>
   </si>
@@ -299,6 +299,9 @@
   </si>
   <si>
     <t>KLD</t>
+  </si>
+  <si>
+    <t>Segment</t>
   </si>
 </sst>
 </file>
@@ -736,164 +739,164 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A38"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>28</v>
       </c>
@@ -906,21 +909,22 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:N100"/>
-  <sheetFormatPr defaultColWidth="9.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.33203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="20.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.28515625" style="3" customWidth="1"/>
-    <col min="5" max="5" width="21.28515625" style="3" customWidth="1"/>
-    <col min="6" max="6" width="6.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="6.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.5" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.5" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.33203125" style="3" customWidth="1"/>
+    <col min="5" max="5" width="21.33203125" style="3" customWidth="1"/>
+    <col min="6" max="6" width="6.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6.6640625" style="3" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="4" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="6.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="20.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>29</v>
       </c>
@@ -957,11 +961,14 @@
       <c r="L1" s="12" t="s">
         <v>85</v>
       </c>
+      <c r="M1" s="12" t="s">
+        <v>87</v>
+      </c>
       <c r="N1" s="12" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="4"/>
       <c r="B2" s="5"/>
       <c r="C2" s="2"/>
@@ -972,7 +979,7 @@
       <c r="I2" s="5"/>
       <c r="J2" s="5"/>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -984,7 +991,7 @@
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -996,7 +1003,7 @@
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -1008,7 +1015,7 @@
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -1020,7 +1027,7 @@
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -1032,7 +1039,7 @@
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -1044,7 +1051,7 @@
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -1056,7 +1063,7 @@
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -1068,7 +1075,7 @@
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -1080,7 +1087,7 @@
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -1092,7 +1099,7 @@
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -1104,7 +1111,7 @@
       <c r="I13" s="2"/>
       <c r="J13" s="2"/>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -1116,7 +1123,7 @@
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -1128,7 +1135,7 @@
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -1140,7 +1147,7 @@
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17" s="2"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -1152,7 +1159,7 @@
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -1164,7 +1171,7 @@
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -1176,7 +1183,7 @@
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -1188,7 +1195,7 @@
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
@@ -1200,7 +1207,7 @@
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
@@ -1212,7 +1219,7 @@
       <c r="I22" s="2"/>
       <c r="J22" s="2"/>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A23" s="2"/>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
@@ -1224,7 +1231,7 @@
       <c r="I23" s="2"/>
       <c r="J23" s="2"/>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
@@ -1236,7 +1243,7 @@
       <c r="I24" s="2"/>
       <c r="J24" s="2"/>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
@@ -1248,7 +1255,7 @@
       <c r="I25" s="2"/>
       <c r="J25" s="2"/>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
@@ -1260,7 +1267,7 @@
       <c r="I26" s="2"/>
       <c r="J26" s="2"/>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
@@ -1272,7 +1279,7 @@
       <c r="I27" s="2"/>
       <c r="J27" s="2"/>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
@@ -1284,7 +1291,7 @@
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
@@ -1296,7 +1303,7 @@
       <c r="I29" s="2"/>
       <c r="J29" s="2"/>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30" s="2"/>
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
@@ -1308,7 +1315,7 @@
       <c r="I30" s="2"/>
       <c r="J30" s="2"/>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
@@ -1320,7 +1327,7 @@
       <c r="I31" s="2"/>
       <c r="J31" s="2"/>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
@@ -1332,7 +1339,7 @@
       <c r="I32" s="2"/>
       <c r="J32" s="2"/>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
@@ -1344,7 +1351,7 @@
       <c r="I33" s="2"/>
       <c r="J33" s="2"/>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
@@ -1356,7 +1363,7 @@
       <c r="I34" s="2"/>
       <c r="J34" s="2"/>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A35" s="2"/>
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
@@ -1368,7 +1375,7 @@
       <c r="I35" s="2"/>
       <c r="J35" s="2"/>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
@@ -1380,7 +1387,7 @@
       <c r="I36" s="2"/>
       <c r="J36" s="2"/>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
@@ -1392,7 +1399,7 @@
       <c r="I37" s="2"/>
       <c r="J37" s="2"/>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A38" s="2"/>
       <c r="B38" s="2"/>
       <c r="C38" s="2"/>
@@ -1404,7 +1411,7 @@
       <c r="I38" s="2"/>
       <c r="J38" s="2"/>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A39" s="2"/>
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
@@ -1416,7 +1423,7 @@
       <c r="I39" s="2"/>
       <c r="J39" s="2"/>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A40" s="2"/>
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
@@ -1428,7 +1435,7 @@
       <c r="I40" s="2"/>
       <c r="J40" s="2"/>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A41" s="2"/>
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
@@ -1440,7 +1447,7 @@
       <c r="I41" s="2"/>
       <c r="J41" s="2"/>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A42" s="2"/>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
@@ -1452,7 +1459,7 @@
       <c r="I42" s="2"/>
       <c r="J42" s="2"/>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A43" s="2"/>
       <c r="B43" s="2"/>
       <c r="C43" s="2"/>
@@ -1464,7 +1471,7 @@
       <c r="I43" s="2"/>
       <c r="J43" s="2"/>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A44" s="2"/>
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
@@ -1476,7 +1483,7 @@
       <c r="I44" s="2"/>
       <c r="J44" s="2"/>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A45" s="2"/>
       <c r="B45" s="2"/>
       <c r="C45" s="2"/>
@@ -1488,7 +1495,7 @@
       <c r="I45" s="2"/>
       <c r="J45" s="2"/>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A46" s="2"/>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
@@ -1500,7 +1507,7 @@
       <c r="I46" s="2"/>
       <c r="J46" s="2"/>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A47" s="2"/>
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
@@ -1512,7 +1519,7 @@
       <c r="I47" s="2"/>
       <c r="J47" s="2"/>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A48" s="2"/>
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
@@ -1524,7 +1531,7 @@
       <c r="I48" s="2"/>
       <c r="J48" s="2"/>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A49" s="2"/>
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
@@ -1536,7 +1543,7 @@
       <c r="I49" s="2"/>
       <c r="J49" s="2"/>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A50" s="2"/>
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
@@ -1548,7 +1555,7 @@
       <c r="I50" s="2"/>
       <c r="J50" s="2"/>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A51" s="2"/>
       <c r="B51" s="2"/>
       <c r="C51" s="2"/>
@@ -1560,7 +1567,7 @@
       <c r="I51" s="2"/>
       <c r="J51" s="2"/>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A52" s="2"/>
       <c r="B52" s="2"/>
       <c r="C52" s="2"/>
@@ -1572,7 +1579,7 @@
       <c r="I52" s="2"/>
       <c r="J52" s="2"/>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A53" s="2"/>
       <c r="B53" s="2"/>
       <c r="C53" s="2"/>
@@ -1584,7 +1591,7 @@
       <c r="I53" s="2"/>
       <c r="J53" s="2"/>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A54" s="2"/>
       <c r="B54" s="2"/>
       <c r="C54" s="2"/>
@@ -1596,7 +1603,7 @@
       <c r="I54" s="2"/>
       <c r="J54" s="2"/>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A55" s="2"/>
       <c r="B55" s="2"/>
       <c r="C55" s="2"/>
@@ -1608,7 +1615,7 @@
       <c r="I55" s="2"/>
       <c r="J55" s="2"/>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A56" s="2"/>
       <c r="B56" s="2"/>
       <c r="C56" s="2"/>
@@ -1620,7 +1627,7 @@
       <c r="I56" s="2"/>
       <c r="J56" s="2"/>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A57" s="2"/>
       <c r="B57" s="2"/>
       <c r="C57" s="2"/>
@@ -1632,7 +1639,7 @@
       <c r="I57" s="2"/>
       <c r="J57" s="2"/>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A58" s="2"/>
       <c r="B58" s="2"/>
       <c r="C58" s="2"/>
@@ -1644,7 +1651,7 @@
       <c r="I58" s="2"/>
       <c r="J58" s="2"/>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A59" s="2"/>
       <c r="B59" s="2"/>
       <c r="C59" s="2"/>
@@ -1656,7 +1663,7 @@
       <c r="I59" s="2"/>
       <c r="J59" s="2"/>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A60" s="2"/>
       <c r="B60" s="2"/>
       <c r="C60" s="2"/>
@@ -1668,7 +1675,7 @@
       <c r="I60" s="2"/>
       <c r="J60" s="2"/>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A61" s="2"/>
       <c r="B61" s="2"/>
       <c r="C61" s="2"/>
@@ -1680,7 +1687,7 @@
       <c r="I61" s="2"/>
       <c r="J61" s="2"/>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A62" s="2"/>
       <c r="B62" s="2"/>
       <c r="C62" s="2"/>
@@ -1692,7 +1699,7 @@
       <c r="I62" s="2"/>
       <c r="J62" s="2"/>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A63" s="2"/>
       <c r="B63" s="2"/>
       <c r="C63" s="2"/>
@@ -1704,7 +1711,7 @@
       <c r="I63" s="2"/>
       <c r="J63" s="2"/>
     </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A64" s="2"/>
       <c r="B64" s="2"/>
       <c r="C64" s="2"/>
@@ -1716,7 +1723,7 @@
       <c r="I64" s="2"/>
       <c r="J64" s="2"/>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A65" s="2"/>
       <c r="B65" s="2"/>
       <c r="C65" s="2"/>
@@ -1728,7 +1735,7 @@
       <c r="I65" s="2"/>
       <c r="J65" s="2"/>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A66" s="2"/>
       <c r="B66" s="2"/>
       <c r="C66" s="2"/>
@@ -1740,7 +1747,7 @@
       <c r="I66" s="2"/>
       <c r="J66" s="2"/>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A67" s="2"/>
       <c r="B67" s="2"/>
       <c r="C67" s="2"/>
@@ -1752,7 +1759,7 @@
       <c r="I67" s="2"/>
       <c r="J67" s="2"/>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A68" s="2"/>
       <c r="B68" s="2"/>
       <c r="C68" s="2"/>
@@ -1764,7 +1771,7 @@
       <c r="I68" s="2"/>
       <c r="J68" s="2"/>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A69" s="2"/>
       <c r="B69" s="2"/>
       <c r="C69" s="2"/>
@@ -1776,7 +1783,7 @@
       <c r="I69" s="2"/>
       <c r="J69" s="2"/>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A70" s="2"/>
       <c r="B70" s="2"/>
       <c r="C70" s="2"/>
@@ -1788,7 +1795,7 @@
       <c r="I70" s="2"/>
       <c r="J70" s="2"/>
     </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A71" s="2"/>
       <c r="B71" s="2"/>
       <c r="C71" s="2"/>
@@ -1800,7 +1807,7 @@
       <c r="I71" s="2"/>
       <c r="J71" s="2"/>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A72" s="2"/>
       <c r="B72" s="2"/>
       <c r="C72" s="2"/>
@@ -1812,7 +1819,7 @@
       <c r="I72" s="2"/>
       <c r="J72" s="2"/>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A73" s="2"/>
       <c r="B73" s="2"/>
       <c r="C73" s="2"/>
@@ -1824,7 +1831,7 @@
       <c r="I73" s="2"/>
       <c r="J73" s="2"/>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A74" s="2"/>
       <c r="B74" s="2"/>
       <c r="C74" s="2"/>
@@ -1836,7 +1843,7 @@
       <c r="I74" s="2"/>
       <c r="J74" s="2"/>
     </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A75" s="2"/>
       <c r="B75" s="2"/>
       <c r="C75" s="2"/>
@@ -1848,7 +1855,7 @@
       <c r="I75" s="2"/>
       <c r="J75" s="2"/>
     </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A76" s="2"/>
       <c r="B76" s="2"/>
       <c r="C76" s="2"/>
@@ -1860,7 +1867,7 @@
       <c r="I76" s="2"/>
       <c r="J76" s="2"/>
     </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A77" s="2"/>
       <c r="B77" s="2"/>
       <c r="C77" s="2"/>
@@ -1872,7 +1879,7 @@
       <c r="I77" s="2"/>
       <c r="J77" s="2"/>
     </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A78" s="2"/>
       <c r="B78" s="2"/>
       <c r="C78" s="2"/>
@@ -1884,7 +1891,7 @@
       <c r="I78" s="2"/>
       <c r="J78" s="2"/>
     </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A79" s="2"/>
       <c r="B79" s="2"/>
       <c r="C79" s="2"/>
@@ -1896,7 +1903,7 @@
       <c r="I79" s="2"/>
       <c r="J79" s="2"/>
     </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A80" s="2"/>
       <c r="B80" s="2"/>
       <c r="C80" s="2"/>
@@ -1908,7 +1915,7 @@
       <c r="I80" s="2"/>
       <c r="J80" s="2"/>
     </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A81" s="2"/>
       <c r="B81" s="2"/>
       <c r="C81" s="2"/>
@@ -1920,7 +1927,7 @@
       <c r="I81" s="2"/>
       <c r="J81" s="2"/>
     </row>
-    <row r="82" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A82" s="2"/>
       <c r="B82" s="2"/>
       <c r="C82" s="2"/>
@@ -1932,7 +1939,7 @@
       <c r="I82" s="2"/>
       <c r="J82" s="2"/>
     </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A83" s="2"/>
       <c r="B83" s="2"/>
       <c r="C83" s="2"/>
@@ -1944,7 +1951,7 @@
       <c r="I83" s="2"/>
       <c r="J83" s="2"/>
     </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A84" s="2"/>
       <c r="B84" s="2"/>
       <c r="C84" s="2"/>
@@ -1956,7 +1963,7 @@
       <c r="I84" s="2"/>
       <c r="J84" s="2"/>
     </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A85" s="2"/>
       <c r="B85" s="2"/>
       <c r="C85" s="2"/>
@@ -1968,7 +1975,7 @@
       <c r="I85" s="2"/>
       <c r="J85" s="2"/>
     </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A86" s="2"/>
       <c r="B86" s="2"/>
       <c r="C86" s="2"/>
@@ -1980,7 +1987,7 @@
       <c r="I86" s="2"/>
       <c r="J86" s="2"/>
     </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A87" s="2"/>
       <c r="B87" s="2"/>
       <c r="C87" s="2"/>
@@ -1992,7 +1999,7 @@
       <c r="I87" s="2"/>
       <c r="J87" s="2"/>
     </row>
-    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A88" s="2"/>
       <c r="B88" s="2"/>
       <c r="C88" s="2"/>
@@ -2004,7 +2011,7 @@
       <c r="I88" s="2"/>
       <c r="J88" s="2"/>
     </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A89" s="2"/>
       <c r="B89" s="2"/>
       <c r="C89" s="2"/>
@@ -2016,7 +2023,7 @@
       <c r="I89" s="2"/>
       <c r="J89" s="2"/>
     </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A90" s="2"/>
       <c r="B90" s="2"/>
       <c r="C90" s="2"/>
@@ -2028,7 +2035,7 @@
       <c r="I90" s="2"/>
       <c r="J90" s="2"/>
     </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A91" s="2"/>
       <c r="B91" s="2"/>
       <c r="C91" s="2"/>
@@ -2040,7 +2047,7 @@
       <c r="I91" s="2"/>
       <c r="J91" s="2"/>
     </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A92" s="2"/>
       <c r="B92" s="2"/>
       <c r="C92" s="2"/>
@@ -2052,7 +2059,7 @@
       <c r="I92" s="2"/>
       <c r="J92" s="2"/>
     </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A93" s="2"/>
       <c r="B93" s="2"/>
       <c r="C93" s="2"/>
@@ -2064,7 +2071,7 @@
       <c r="I93" s="2"/>
       <c r="J93" s="2"/>
     </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A94" s="2"/>
       <c r="B94" s="2"/>
       <c r="C94" s="2"/>
@@ -2076,7 +2083,7 @@
       <c r="I94" s="2"/>
       <c r="J94" s="2"/>
     </row>
-    <row r="95" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A95" s="2"/>
       <c r="B95" s="2"/>
       <c r="C95" s="2"/>
@@ -2088,7 +2095,7 @@
       <c r="I95" s="2"/>
       <c r="J95" s="2"/>
     </row>
-    <row r="96" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A96" s="2"/>
       <c r="B96" s="2"/>
       <c r="C96" s="2"/>
@@ -2100,7 +2107,7 @@
       <c r="I96" s="2"/>
       <c r="J96" s="2"/>
     </row>
-    <row r="97" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A97" s="2"/>
       <c r="B97" s="2"/>
       <c r="C97" s="2"/>
@@ -2112,7 +2119,7 @@
       <c r="I97" s="2"/>
       <c r="J97" s="2"/>
     </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A98" s="2"/>
       <c r="B98" s="2"/>
       <c r="C98" s="2"/>
@@ -2124,7 +2131,7 @@
       <c r="I98" s="2"/>
       <c r="J98" s="2"/>
     </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A99" s="2"/>
       <c r="B99" s="2"/>
       <c r="C99" s="2"/>
@@ -2136,7 +2143,7 @@
       <c r="I99" s="2"/>
       <c r="J99" s="2"/>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A100" s="2"/>
       <c r="B100" s="2"/>
       <c r="C100" s="2"/>
@@ -2180,14 +2187,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:Q100"/>
-  <sheetFormatPr defaultColWidth="9.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.33203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="22.28515625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="6.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="17" width="20.7109375" style="3" customWidth="1"/>
+    <col min="1" max="1" width="22.33203125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="6.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="17" width="20.6640625" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="12" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" s="12" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>29</v>
       </c>
@@ -2240,7 +2247,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A2" s="4"/>
       <c r="D2" s="2"/>
       <c r="E2" s="5"/>
@@ -2257,7 +2264,7 @@
       <c r="P2" s="2"/>
       <c r="Q2" s="2"/>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
@@ -2275,7 +2282,7 @@
       <c r="P3" s="2"/>
       <c r="Q3" s="2"/>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
@@ -2293,7 +2300,7 @@
       <c r="P4" s="2"/>
       <c r="Q4" s="2"/>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
@@ -2311,7 +2318,7 @@
       <c r="P5" s="2"/>
       <c r="Q5" s="2"/>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
@@ -2329,7 +2336,7 @@
       <c r="P6" s="2"/>
       <c r="Q6" s="2"/>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
@@ -2347,7 +2354,7 @@
       <c r="P7" s="2"/>
       <c r="Q7" s="2"/>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
@@ -2365,7 +2372,7 @@
       <c r="P8" s="2"/>
       <c r="Q8" s="2"/>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
@@ -2383,7 +2390,7 @@
       <c r="P9" s="2"/>
       <c r="Q9" s="2"/>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
@@ -2401,7 +2408,7 @@
       <c r="P10" s="2"/>
       <c r="Q10" s="2"/>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
@@ -2419,7 +2426,7 @@
       <c r="P11" s="2"/>
       <c r="Q11" s="2"/>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
@@ -2437,7 +2444,7 @@
       <c r="P12" s="2"/>
       <c r="Q12" s="2"/>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
@@ -2455,7 +2462,7 @@
       <c r="P13" s="2"/>
       <c r="Q13" s="2"/>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
@@ -2473,7 +2480,7 @@
       <c r="P14" s="2"/>
       <c r="Q14" s="2"/>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
@@ -2491,7 +2498,7 @@
       <c r="P15" s="2"/>
       <c r="Q15" s="2"/>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
@@ -2509,7 +2516,7 @@
       <c r="P16" s="2"/>
       <c r="Q16" s="2"/>
     </row>
-    <row r="17" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
@@ -2527,7 +2534,7 @@
       <c r="P17" s="2"/>
       <c r="Q17" s="2"/>
     </row>
-    <row r="18" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
@@ -2545,7 +2552,7 @@
       <c r="P18" s="2"/>
       <c r="Q18" s="2"/>
     </row>
-    <row r="19" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
@@ -2563,7 +2570,7 @@
       <c r="P19" s="2"/>
       <c r="Q19" s="2"/>
     </row>
-    <row r="20" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
@@ -2581,7 +2588,7 @@
       <c r="P20" s="2"/>
       <c r="Q20" s="2"/>
     </row>
-    <row r="21" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
@@ -2599,7 +2606,7 @@
       <c r="P21" s="2"/>
       <c r="Q21" s="2"/>
     </row>
-    <row r="22" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
@@ -2617,7 +2624,7 @@
       <c r="P22" s="2"/>
       <c r="Q22" s="2"/>
     </row>
-    <row r="23" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
@@ -2635,7 +2642,7 @@
       <c r="P23" s="2"/>
       <c r="Q23" s="2"/>
     </row>
-    <row r="24" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
@@ -2653,7 +2660,7 @@
       <c r="P24" s="2"/>
       <c r="Q24" s="2"/>
     </row>
-    <row r="25" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
@@ -2671,7 +2678,7 @@
       <c r="P25" s="2"/>
       <c r="Q25" s="2"/>
     </row>
-    <row r="26" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
       <c r="D26" s="2"/>
@@ -2689,7 +2696,7 @@
       <c r="P26" s="2"/>
       <c r="Q26" s="2"/>
     </row>
-    <row r="27" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
       <c r="D27" s="2"/>
@@ -2707,7 +2714,7 @@
       <c r="P27" s="2"/>
       <c r="Q27" s="2"/>
     </row>
-    <row r="28" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
       <c r="D28" s="2"/>
@@ -2725,7 +2732,7 @@
       <c r="P28" s="2"/>
       <c r="Q28" s="2"/>
     </row>
-    <row r="29" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
       <c r="D29" s="2"/>
@@ -2743,7 +2750,7 @@
       <c r="P29" s="2"/>
       <c r="Q29" s="2"/>
     </row>
-    <row r="30" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
@@ -2761,7 +2768,7 @@
       <c r="P30" s="2"/>
       <c r="Q30" s="2"/>
     </row>
-    <row r="31" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
       <c r="D31" s="2"/>
@@ -2779,7 +2786,7 @@
       <c r="P31" s="2"/>
       <c r="Q31" s="2"/>
     </row>
-    <row r="32" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
       <c r="D32" s="2"/>
@@ -2797,7 +2804,7 @@
       <c r="P32" s="2"/>
       <c r="Q32" s="2"/>
     </row>
-    <row r="33" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
@@ -2815,7 +2822,7 @@
       <c r="P33" s="2"/>
       <c r="Q33" s="2"/>
     </row>
-    <row r="34" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
@@ -2833,7 +2840,7 @@
       <c r="P34" s="2"/>
       <c r="Q34" s="2"/>
     </row>
-    <row r="35" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
@@ -2851,7 +2858,7 @@
       <c r="P35" s="2"/>
       <c r="Q35" s="2"/>
     </row>
-    <row r="36" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
@@ -2869,7 +2876,7 @@
       <c r="P36" s="2"/>
       <c r="Q36" s="2"/>
     </row>
-    <row r="37" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
@@ -2887,7 +2894,7 @@
       <c r="P37" s="2"/>
       <c r="Q37" s="2"/>
     </row>
-    <row r="38" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B38" s="2"/>
       <c r="C38" s="2"/>
       <c r="D38" s="2"/>
@@ -2905,7 +2912,7 @@
       <c r="P38" s="2"/>
       <c r="Q38" s="2"/>
     </row>
-    <row r="39" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
       <c r="D39" s="2"/>
@@ -2923,7 +2930,7 @@
       <c r="P39" s="2"/>
       <c r="Q39" s="2"/>
     </row>
-    <row r="40" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
       <c r="D40" s="2"/>
@@ -2941,7 +2948,7 @@
       <c r="P40" s="2"/>
       <c r="Q40" s="2"/>
     </row>
-    <row r="41" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
       <c r="D41" s="2"/>
@@ -2959,7 +2966,7 @@
       <c r="P41" s="2"/>
       <c r="Q41" s="2"/>
     </row>
-    <row r="42" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
       <c r="D42" s="2"/>
@@ -2977,7 +2984,7 @@
       <c r="P42" s="2"/>
       <c r="Q42" s="2"/>
     </row>
-    <row r="43" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B43" s="2"/>
       <c r="C43" s="2"/>
       <c r="D43" s="2"/>
@@ -2995,7 +3002,7 @@
       <c r="P43" s="2"/>
       <c r="Q43" s="2"/>
     </row>
-    <row r="44" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
       <c r="D44" s="2"/>
@@ -3013,7 +3020,7 @@
       <c r="P44" s="2"/>
       <c r="Q44" s="2"/>
     </row>
-    <row r="45" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B45" s="2"/>
       <c r="C45" s="2"/>
       <c r="D45" s="2"/>
@@ -3031,7 +3038,7 @@
       <c r="P45" s="2"/>
       <c r="Q45" s="2"/>
     </row>
-    <row r="46" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
       <c r="D46" s="2"/>
@@ -3049,7 +3056,7 @@
       <c r="P46" s="2"/>
       <c r="Q46" s="2"/>
     </row>
-    <row r="47" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
       <c r="D47" s="2"/>
@@ -3067,7 +3074,7 @@
       <c r="P47" s="2"/>
       <c r="Q47" s="2"/>
     </row>
-    <row r="48" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
       <c r="D48" s="2"/>
@@ -3085,7 +3092,7 @@
       <c r="P48" s="2"/>
       <c r="Q48" s="2"/>
     </row>
-    <row r="49" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
       <c r="D49" s="2"/>
@@ -3103,7 +3110,7 @@
       <c r="P49" s="2"/>
       <c r="Q49" s="2"/>
     </row>
-    <row r="50" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
       <c r="D50" s="2"/>
@@ -3121,7 +3128,7 @@
       <c r="P50" s="2"/>
       <c r="Q50" s="2"/>
     </row>
-    <row r="51" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B51" s="2"/>
       <c r="C51" s="2"/>
       <c r="D51" s="2"/>
@@ -3139,7 +3146,7 @@
       <c r="P51" s="2"/>
       <c r="Q51" s="2"/>
     </row>
-    <row r="52" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B52" s="2"/>
       <c r="C52" s="2"/>
       <c r="D52" s="2"/>
@@ -3157,7 +3164,7 @@
       <c r="P52" s="2"/>
       <c r="Q52" s="2"/>
     </row>
-    <row r="53" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B53" s="2"/>
       <c r="C53" s="2"/>
       <c r="D53" s="2"/>
@@ -3175,7 +3182,7 @@
       <c r="P53" s="2"/>
       <c r="Q53" s="2"/>
     </row>
-    <row r="54" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B54" s="2"/>
       <c r="C54" s="2"/>
       <c r="D54" s="2"/>
@@ -3193,7 +3200,7 @@
       <c r="P54" s="2"/>
       <c r="Q54" s="2"/>
     </row>
-    <row r="55" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B55" s="2"/>
       <c r="C55" s="2"/>
       <c r="D55" s="2"/>
@@ -3211,7 +3218,7 @@
       <c r="P55" s="2"/>
       <c r="Q55" s="2"/>
     </row>
-    <row r="56" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B56" s="2"/>
       <c r="C56" s="2"/>
       <c r="D56" s="2"/>
@@ -3229,7 +3236,7 @@
       <c r="P56" s="2"/>
       <c r="Q56" s="2"/>
     </row>
-    <row r="57" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B57" s="2"/>
       <c r="C57" s="2"/>
       <c r="D57" s="2"/>
@@ -3247,7 +3254,7 @@
       <c r="P57" s="2"/>
       <c r="Q57" s="2"/>
     </row>
-    <row r="58" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B58" s="2"/>
       <c r="C58" s="2"/>
       <c r="D58" s="2"/>
@@ -3265,7 +3272,7 @@
       <c r="P58" s="2"/>
       <c r="Q58" s="2"/>
     </row>
-    <row r="59" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B59" s="2"/>
       <c r="C59" s="2"/>
       <c r="D59" s="2"/>
@@ -3283,7 +3290,7 @@
       <c r="P59" s="2"/>
       <c r="Q59" s="2"/>
     </row>
-    <row r="60" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B60" s="2"/>
       <c r="C60" s="2"/>
       <c r="D60" s="2"/>
@@ -3301,7 +3308,7 @@
       <c r="P60" s="2"/>
       <c r="Q60" s="2"/>
     </row>
-    <row r="61" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B61" s="2"/>
       <c r="C61" s="2"/>
       <c r="D61" s="2"/>
@@ -3319,7 +3326,7 @@
       <c r="P61" s="2"/>
       <c r="Q61" s="2"/>
     </row>
-    <row r="62" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B62" s="2"/>
       <c r="C62" s="2"/>
       <c r="D62" s="2"/>
@@ -3337,7 +3344,7 @@
       <c r="P62" s="2"/>
       <c r="Q62" s="2"/>
     </row>
-    <row r="63" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B63" s="2"/>
       <c r="C63" s="2"/>
       <c r="D63" s="2"/>
@@ -3355,7 +3362,7 @@
       <c r="P63" s="2"/>
       <c r="Q63" s="2"/>
     </row>
-    <row r="64" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B64" s="2"/>
       <c r="C64" s="2"/>
       <c r="D64" s="2"/>
@@ -3373,7 +3380,7 @@
       <c r="P64" s="2"/>
       <c r="Q64" s="2"/>
     </row>
-    <row r="65" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B65" s="2"/>
       <c r="C65" s="2"/>
       <c r="D65" s="2"/>
@@ -3391,7 +3398,7 @@
       <c r="P65" s="2"/>
       <c r="Q65" s="2"/>
     </row>
-    <row r="66" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B66" s="2"/>
       <c r="C66" s="2"/>
       <c r="D66" s="2"/>
@@ -3409,7 +3416,7 @@
       <c r="P66" s="2"/>
       <c r="Q66" s="2"/>
     </row>
-    <row r="67" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B67" s="2"/>
       <c r="C67" s="2"/>
       <c r="D67" s="2"/>
@@ -3427,7 +3434,7 @@
       <c r="P67" s="2"/>
       <c r="Q67" s="2"/>
     </row>
-    <row r="68" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B68" s="2"/>
       <c r="C68" s="2"/>
       <c r="D68" s="2"/>
@@ -3445,7 +3452,7 @@
       <c r="P68" s="2"/>
       <c r="Q68" s="2"/>
     </row>
-    <row r="69" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B69" s="2"/>
       <c r="C69" s="2"/>
       <c r="D69" s="2"/>
@@ -3463,7 +3470,7 @@
       <c r="P69" s="2"/>
       <c r="Q69" s="2"/>
     </row>
-    <row r="70" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B70" s="2"/>
       <c r="C70" s="2"/>
       <c r="D70" s="2"/>
@@ -3481,7 +3488,7 @@
       <c r="P70" s="2"/>
       <c r="Q70" s="2"/>
     </row>
-    <row r="71" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B71" s="2"/>
       <c r="C71" s="2"/>
       <c r="D71" s="2"/>
@@ -3499,7 +3506,7 @@
       <c r="P71" s="2"/>
       <c r="Q71" s="2"/>
     </row>
-    <row r="72" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B72" s="2"/>
       <c r="C72" s="2"/>
       <c r="D72" s="2"/>
@@ -3517,7 +3524,7 @@
       <c r="P72" s="2"/>
       <c r="Q72" s="2"/>
     </row>
-    <row r="73" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B73" s="2"/>
       <c r="C73" s="2"/>
       <c r="D73" s="2"/>
@@ -3535,7 +3542,7 @@
       <c r="P73" s="2"/>
       <c r="Q73" s="2"/>
     </row>
-    <row r="74" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="74" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B74" s="2"/>
       <c r="C74" s="2"/>
       <c r="D74" s="2"/>
@@ -3553,7 +3560,7 @@
       <c r="P74" s="2"/>
       <c r="Q74" s="2"/>
     </row>
-    <row r="75" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="75" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B75" s="2"/>
       <c r="C75" s="2"/>
       <c r="D75" s="2"/>
@@ -3571,7 +3578,7 @@
       <c r="P75" s="2"/>
       <c r="Q75" s="2"/>
     </row>
-    <row r="76" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="76" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B76" s="2"/>
       <c r="C76" s="2"/>
       <c r="D76" s="2"/>
@@ -3589,7 +3596,7 @@
       <c r="P76" s="2"/>
       <c r="Q76" s="2"/>
     </row>
-    <row r="77" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B77" s="2"/>
       <c r="C77" s="2"/>
       <c r="D77" s="2"/>
@@ -3607,7 +3614,7 @@
       <c r="P77" s="2"/>
       <c r="Q77" s="2"/>
     </row>
-    <row r="78" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="78" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B78" s="2"/>
       <c r="C78" s="2"/>
       <c r="D78" s="2"/>
@@ -3625,7 +3632,7 @@
       <c r="P78" s="2"/>
       <c r="Q78" s="2"/>
     </row>
-    <row r="79" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="79" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B79" s="2"/>
       <c r="C79" s="2"/>
       <c r="D79" s="2"/>
@@ -3643,7 +3650,7 @@
       <c r="P79" s="2"/>
       <c r="Q79" s="2"/>
     </row>
-    <row r="80" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="80" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B80" s="2"/>
       <c r="C80" s="2"/>
       <c r="D80" s="2"/>
@@ -3661,7 +3668,7 @@
       <c r="P80" s="2"/>
       <c r="Q80" s="2"/>
     </row>
-    <row r="81" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B81" s="2"/>
       <c r="C81" s="2"/>
       <c r="D81" s="2"/>
@@ -3679,7 +3686,7 @@
       <c r="P81" s="2"/>
       <c r="Q81" s="2"/>
     </row>
-    <row r="82" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B82" s="2"/>
       <c r="C82" s="2"/>
       <c r="D82" s="2"/>
@@ -3697,7 +3704,7 @@
       <c r="P82" s="2"/>
       <c r="Q82" s="2"/>
     </row>
-    <row r="83" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="83" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B83" s="2"/>
       <c r="C83" s="2"/>
       <c r="D83" s="2"/>
@@ -3715,7 +3722,7 @@
       <c r="P83" s="2"/>
       <c r="Q83" s="2"/>
     </row>
-    <row r="84" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="84" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B84" s="2"/>
       <c r="C84" s="2"/>
       <c r="D84" s="2"/>
@@ -3733,7 +3740,7 @@
       <c r="P84" s="2"/>
       <c r="Q84" s="2"/>
     </row>
-    <row r="85" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="85" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B85" s="2"/>
       <c r="C85" s="2"/>
       <c r="D85" s="2"/>
@@ -3751,7 +3758,7 @@
       <c r="P85" s="2"/>
       <c r="Q85" s="2"/>
     </row>
-    <row r="86" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="86" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B86" s="2"/>
       <c r="C86" s="2"/>
       <c r="D86" s="2"/>
@@ -3769,7 +3776,7 @@
       <c r="P86" s="2"/>
       <c r="Q86" s="2"/>
     </row>
-    <row r="87" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="87" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B87" s="2"/>
       <c r="C87" s="2"/>
       <c r="D87" s="2"/>
@@ -3787,7 +3794,7 @@
       <c r="P87" s="2"/>
       <c r="Q87" s="2"/>
     </row>
-    <row r="88" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="88" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B88" s="2"/>
       <c r="C88" s="2"/>
       <c r="D88" s="2"/>
@@ -3805,7 +3812,7 @@
       <c r="P88" s="2"/>
       <c r="Q88" s="2"/>
     </row>
-    <row r="89" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="89" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B89" s="2"/>
       <c r="C89" s="2"/>
       <c r="D89" s="2"/>
@@ -3823,7 +3830,7 @@
       <c r="P89" s="2"/>
       <c r="Q89" s="2"/>
     </row>
-    <row r="90" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="90" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B90" s="2"/>
       <c r="C90" s="2"/>
       <c r="D90" s="2"/>
@@ -3841,7 +3848,7 @@
       <c r="P90" s="2"/>
       <c r="Q90" s="2"/>
     </row>
-    <row r="91" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="91" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B91" s="2"/>
       <c r="C91" s="2"/>
       <c r="D91" s="2"/>
@@ -3859,7 +3866,7 @@
       <c r="P91" s="2"/>
       <c r="Q91" s="2"/>
     </row>
-    <row r="92" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="92" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B92" s="2"/>
       <c r="C92" s="2"/>
       <c r="D92" s="2"/>
@@ -3877,7 +3884,7 @@
       <c r="P92" s="2"/>
       <c r="Q92" s="2"/>
     </row>
-    <row r="93" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="93" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B93" s="2"/>
       <c r="C93" s="2"/>
       <c r="D93" s="2"/>
@@ -3895,7 +3902,7 @@
       <c r="P93" s="2"/>
       <c r="Q93" s="2"/>
     </row>
-    <row r="94" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="94" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B94" s="2"/>
       <c r="C94" s="2"/>
       <c r="D94" s="2"/>
@@ -3913,7 +3920,7 @@
       <c r="P94" s="2"/>
       <c r="Q94" s="2"/>
     </row>
-    <row r="95" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="95" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B95" s="2"/>
       <c r="C95" s="2"/>
       <c r="D95" s="2"/>
@@ -3931,7 +3938,7 @@
       <c r="P95" s="2"/>
       <c r="Q95" s="2"/>
     </row>
-    <row r="96" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="96" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B96" s="2"/>
       <c r="C96" s="2"/>
       <c r="D96" s="2"/>
@@ -3949,7 +3956,7 @@
       <c r="P96" s="2"/>
       <c r="Q96" s="2"/>
     </row>
-    <row r="97" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="97" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B97" s="2"/>
       <c r="C97" s="2"/>
       <c r="D97" s="2"/>
@@ -3967,7 +3974,7 @@
       <c r="P97" s="2"/>
       <c r="Q97" s="2"/>
     </row>
-    <row r="98" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="98" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B98" s="2"/>
       <c r="C98" s="2"/>
       <c r="D98" s="2"/>
@@ -3985,7 +3992,7 @@
       <c r="P98" s="2"/>
       <c r="Q98" s="2"/>
     </row>
-    <row r="99" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="99" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B99" s="2"/>
       <c r="C99" s="2"/>
       <c r="D99" s="2"/>
@@ -4003,7 +4010,7 @@
       <c r="P99" s="2"/>
       <c r="Q99" s="2"/>
     </row>
-    <row r="100" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="100" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B100" s="2"/>
       <c r="C100" s="2"/>
       <c r="D100" s="2"/>
@@ -4048,24 +4055,24 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:M100"/>
-  <sheetFormatPr defaultColWidth="9.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.33203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="22.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.5703125" style="3" customWidth="1"/>
-    <col min="6" max="6" width="8.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.5" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.5" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.5" style="3" customWidth="1"/>
+    <col min="6" max="6" width="8.5" style="3" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="6" style="3" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="8" style="3" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="8" style="3" customWidth="1"/>
     <col min="10" max="10" width="12" style="3" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.5" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.6640625" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>29</v>
       </c>
@@ -4106,7 +4113,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" s="4"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
@@ -4117,7 +4124,7 @@
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" s="4"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -4129,7 +4136,7 @@
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" s="4"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -4141,7 +4148,7 @@
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" s="4"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -4153,7 +4160,7 @@
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" s="4"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -4165,7 +4172,7 @@
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" s="4"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -4177,7 +4184,7 @@
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="4"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -4189,7 +4196,7 @@
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="4"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -4201,7 +4208,7 @@
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="4"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -4213,7 +4220,7 @@
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="4"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -4225,7 +4232,7 @@
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="9"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -4237,7 +4244,7 @@
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" s="9"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -4249,7 +4256,7 @@
       <c r="I13" s="2"/>
       <c r="J13" s="2"/>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" s="9"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -4261,7 +4268,7 @@
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" s="9"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -4273,7 +4280,7 @@
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="9"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -4285,7 +4292,7 @@
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17" s="9"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -4297,7 +4304,7 @@
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="9"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -4309,7 +4316,7 @@
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" s="9"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -4321,7 +4328,7 @@
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" s="9"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -4333,7 +4340,7 @@
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" s="9"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
@@ -4345,7 +4352,7 @@
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
@@ -4357,7 +4364,7 @@
       <c r="I22" s="2"/>
       <c r="J22" s="2"/>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A23" s="2"/>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
@@ -4369,7 +4376,7 @@
       <c r="I23" s="2"/>
       <c r="J23" s="2"/>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
@@ -4381,7 +4388,7 @@
       <c r="I24" s="2"/>
       <c r="J24" s="2"/>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
@@ -4393,7 +4400,7 @@
       <c r="I25" s="2"/>
       <c r="J25" s="2"/>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
@@ -4405,7 +4412,7 @@
       <c r="I26" s="2"/>
       <c r="J26" s="2"/>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
@@ -4417,7 +4424,7 @@
       <c r="I27" s="2"/>
       <c r="J27" s="2"/>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
@@ -4429,7 +4436,7 @@
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
@@ -4441,7 +4448,7 @@
       <c r="I29" s="2"/>
       <c r="J29" s="2"/>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30" s="2"/>
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
@@ -4453,7 +4460,7 @@
       <c r="I30" s="2"/>
       <c r="J30" s="2"/>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
@@ -4465,7 +4472,7 @@
       <c r="I31" s="2"/>
       <c r="J31" s="2"/>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
@@ -4477,7 +4484,7 @@
       <c r="I32" s="2"/>
       <c r="J32" s="2"/>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
@@ -4489,7 +4496,7 @@
       <c r="I33" s="2"/>
       <c r="J33" s="2"/>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
@@ -4501,7 +4508,7 @@
       <c r="I34" s="2"/>
       <c r="J34" s="2"/>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A35" s="2"/>
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
@@ -4513,7 +4520,7 @@
       <c r="I35" s="2"/>
       <c r="J35" s="2"/>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
@@ -4525,7 +4532,7 @@
       <c r="I36" s="2"/>
       <c r="J36" s="2"/>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
@@ -4537,7 +4544,7 @@
       <c r="I37" s="2"/>
       <c r="J37" s="2"/>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A38" s="2"/>
       <c r="B38" s="2"/>
       <c r="C38" s="2"/>
@@ -4549,7 +4556,7 @@
       <c r="I38" s="2"/>
       <c r="J38" s="2"/>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A39" s="2"/>
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
@@ -4561,7 +4568,7 @@
       <c r="I39" s="2"/>
       <c r="J39" s="2"/>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A40" s="2"/>
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
@@ -4573,7 +4580,7 @@
       <c r="I40" s="2"/>
       <c r="J40" s="2"/>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A41" s="2"/>
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
@@ -4585,7 +4592,7 @@
       <c r="I41" s="2"/>
       <c r="J41" s="2"/>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A42" s="2"/>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
@@ -4597,7 +4604,7 @@
       <c r="I42" s="2"/>
       <c r="J42" s="2"/>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A43" s="2"/>
       <c r="B43" s="2"/>
       <c r="C43" s="2"/>
@@ -4609,7 +4616,7 @@
       <c r="I43" s="2"/>
       <c r="J43" s="2"/>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A44" s="2"/>
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
@@ -4621,7 +4628,7 @@
       <c r="I44" s="2"/>
       <c r="J44" s="2"/>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A45" s="2"/>
       <c r="B45" s="2"/>
       <c r="C45" s="2"/>
@@ -4633,7 +4640,7 @@
       <c r="I45" s="2"/>
       <c r="J45" s="2"/>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A46" s="2"/>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
@@ -4645,7 +4652,7 @@
       <c r="I46" s="2"/>
       <c r="J46" s="2"/>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A47" s="2"/>
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
@@ -4657,7 +4664,7 @@
       <c r="I47" s="2"/>
       <c r="J47" s="2"/>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A48" s="2"/>
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
@@ -4669,7 +4676,7 @@
       <c r="I48" s="2"/>
       <c r="J48" s="2"/>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A49" s="2"/>
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
@@ -4681,7 +4688,7 @@
       <c r="I49" s="2"/>
       <c r="J49" s="2"/>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A50" s="2"/>
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
@@ -4693,7 +4700,7 @@
       <c r="I50" s="2"/>
       <c r="J50" s="2"/>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A51" s="2"/>
       <c r="B51" s="2"/>
       <c r="C51" s="2"/>
@@ -4705,7 +4712,7 @@
       <c r="I51" s="2"/>
       <c r="J51" s="2"/>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A52" s="2"/>
       <c r="B52" s="2"/>
       <c r="C52" s="2"/>
@@ -4717,7 +4724,7 @@
       <c r="I52" s="2"/>
       <c r="J52" s="2"/>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A53" s="2"/>
       <c r="B53" s="2"/>
       <c r="C53" s="2"/>
@@ -4729,7 +4736,7 @@
       <c r="I53" s="2"/>
       <c r="J53" s="2"/>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A54" s="2"/>
       <c r="B54" s="2"/>
       <c r="C54" s="2"/>
@@ -4741,7 +4748,7 @@
       <c r="I54" s="2"/>
       <c r="J54" s="2"/>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A55" s="2"/>
       <c r="B55" s="2"/>
       <c r="C55" s="2"/>
@@ -4753,7 +4760,7 @@
       <c r="I55" s="2"/>
       <c r="J55" s="2"/>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A56" s="2"/>
       <c r="B56" s="2"/>
       <c r="C56" s="2"/>
@@ -4765,7 +4772,7 @@
       <c r="I56" s="2"/>
       <c r="J56" s="2"/>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A57" s="2"/>
       <c r="B57" s="2"/>
       <c r="C57" s="2"/>
@@ -4777,7 +4784,7 @@
       <c r="I57" s="2"/>
       <c r="J57" s="2"/>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A58" s="2"/>
       <c r="B58" s="2"/>
       <c r="C58" s="2"/>
@@ -4789,7 +4796,7 @@
       <c r="I58" s="2"/>
       <c r="J58" s="2"/>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A59" s="2"/>
       <c r="B59" s="2"/>
       <c r="C59" s="2"/>
@@ -4801,7 +4808,7 @@
       <c r="I59" s="2"/>
       <c r="J59" s="2"/>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A60" s="2"/>
       <c r="B60" s="2"/>
       <c r="C60" s="2"/>
@@ -4813,7 +4820,7 @@
       <c r="I60" s="2"/>
       <c r="J60" s="2"/>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A61" s="2"/>
       <c r="B61" s="2"/>
       <c r="C61" s="2"/>
@@ -4825,7 +4832,7 @@
       <c r="I61" s="2"/>
       <c r="J61" s="2"/>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A62" s="2"/>
       <c r="B62" s="2"/>
       <c r="C62" s="2"/>
@@ -4837,7 +4844,7 @@
       <c r="I62" s="2"/>
       <c r="J62" s="2"/>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A63" s="2"/>
       <c r="B63" s="2"/>
       <c r="C63" s="2"/>
@@ -4849,7 +4856,7 @@
       <c r="I63" s="2"/>
       <c r="J63" s="2"/>
     </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A64" s="2"/>
       <c r="B64" s="2"/>
       <c r="C64" s="2"/>
@@ -4861,7 +4868,7 @@
       <c r="I64" s="2"/>
       <c r="J64" s="2"/>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A65" s="2"/>
       <c r="B65" s="2"/>
       <c r="C65" s="2"/>
@@ -4873,7 +4880,7 @@
       <c r="I65" s="2"/>
       <c r="J65" s="2"/>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A66" s="2"/>
       <c r="B66" s="2"/>
       <c r="C66" s="2"/>
@@ -4885,7 +4892,7 @@
       <c r="I66" s="2"/>
       <c r="J66" s="2"/>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A67" s="2"/>
       <c r="B67" s="2"/>
       <c r="C67" s="2"/>
@@ -4897,7 +4904,7 @@
       <c r="I67" s="2"/>
       <c r="J67" s="2"/>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A68" s="2"/>
       <c r="B68" s="2"/>
       <c r="C68" s="2"/>
@@ -4909,7 +4916,7 @@
       <c r="I68" s="2"/>
       <c r="J68" s="2"/>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A69" s="2"/>
       <c r="B69" s="2"/>
       <c r="C69" s="2"/>
@@ -4921,7 +4928,7 @@
       <c r="I69" s="2"/>
       <c r="J69" s="2"/>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A70" s="2"/>
       <c r="B70" s="2"/>
       <c r="C70" s="2"/>
@@ -4933,7 +4940,7 @@
       <c r="I70" s="2"/>
       <c r="J70" s="2"/>
     </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A71" s="2"/>
       <c r="B71" s="2"/>
       <c r="C71" s="2"/>
@@ -4945,7 +4952,7 @@
       <c r="I71" s="2"/>
       <c r="J71" s="2"/>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A72" s="2"/>
       <c r="B72" s="2"/>
       <c r="C72" s="2"/>
@@ -4957,7 +4964,7 @@
       <c r="I72" s="2"/>
       <c r="J72" s="2"/>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A73" s="2"/>
       <c r="B73" s="2"/>
       <c r="C73" s="2"/>
@@ -4969,7 +4976,7 @@
       <c r="I73" s="2"/>
       <c r="J73" s="2"/>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A74" s="2"/>
       <c r="B74" s="2"/>
       <c r="C74" s="2"/>
@@ -4981,7 +4988,7 @@
       <c r="I74" s="2"/>
       <c r="J74" s="2"/>
     </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A75" s="2"/>
       <c r="B75" s="2"/>
       <c r="C75" s="2"/>
@@ -4993,7 +5000,7 @@
       <c r="I75" s="2"/>
       <c r="J75" s="2"/>
     </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A76" s="2"/>
       <c r="B76" s="2"/>
       <c r="C76" s="2"/>
@@ -5005,7 +5012,7 @@
       <c r="I76" s="2"/>
       <c r="J76" s="2"/>
     </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A77" s="2"/>
       <c r="B77" s="2"/>
       <c r="C77" s="2"/>
@@ -5017,7 +5024,7 @@
       <c r="I77" s="2"/>
       <c r="J77" s="2"/>
     </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A78" s="2"/>
       <c r="B78" s="2"/>
       <c r="C78" s="2"/>
@@ -5029,7 +5036,7 @@
       <c r="I78" s="2"/>
       <c r="J78" s="2"/>
     </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A79" s="2"/>
       <c r="B79" s="2"/>
       <c r="C79" s="2"/>
@@ -5041,7 +5048,7 @@
       <c r="I79" s="2"/>
       <c r="J79" s="2"/>
     </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A80" s="2"/>
       <c r="B80" s="2"/>
       <c r="C80" s="2"/>
@@ -5053,7 +5060,7 @@
       <c r="I80" s="2"/>
       <c r="J80" s="2"/>
     </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A81" s="2"/>
       <c r="B81" s="2"/>
       <c r="C81" s="2"/>
@@ -5065,7 +5072,7 @@
       <c r="I81" s="2"/>
       <c r="J81" s="2"/>
     </row>
-    <row r="82" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A82" s="2"/>
       <c r="B82" s="2"/>
       <c r="C82" s="2"/>
@@ -5077,7 +5084,7 @@
       <c r="I82" s="2"/>
       <c r="J82" s="2"/>
     </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A83" s="2"/>
       <c r="B83" s="2"/>
       <c r="C83" s="2"/>
@@ -5089,7 +5096,7 @@
       <c r="I83" s="2"/>
       <c r="J83" s="2"/>
     </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A84" s="2"/>
       <c r="B84" s="2"/>
       <c r="C84" s="2"/>
@@ -5101,7 +5108,7 @@
       <c r="I84" s="2"/>
       <c r="J84" s="2"/>
     </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A85" s="2"/>
       <c r="B85" s="2"/>
       <c r="C85" s="2"/>
@@ -5113,7 +5120,7 @@
       <c r="I85" s="2"/>
       <c r="J85" s="2"/>
     </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A86" s="2"/>
       <c r="B86" s="2"/>
       <c r="C86" s="2"/>
@@ -5125,7 +5132,7 @@
       <c r="I86" s="2"/>
       <c r="J86" s="2"/>
     </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A87" s="2"/>
       <c r="B87" s="2"/>
       <c r="C87" s="2"/>
@@ -5137,7 +5144,7 @@
       <c r="I87" s="2"/>
       <c r="J87" s="2"/>
     </row>
-    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A88" s="2"/>
       <c r="B88" s="2"/>
       <c r="C88" s="2"/>
@@ -5149,7 +5156,7 @@
       <c r="I88" s="2"/>
       <c r="J88" s="2"/>
     </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A89" s="2"/>
       <c r="B89" s="2"/>
       <c r="C89" s="2"/>
@@ -5161,7 +5168,7 @@
       <c r="I89" s="2"/>
       <c r="J89" s="2"/>
     </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A90" s="2"/>
       <c r="B90" s="2"/>
       <c r="C90" s="2"/>
@@ -5173,7 +5180,7 @@
       <c r="I90" s="2"/>
       <c r="J90" s="2"/>
     </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A91" s="2"/>
       <c r="B91" s="2"/>
       <c r="C91" s="2"/>
@@ -5185,7 +5192,7 @@
       <c r="I91" s="2"/>
       <c r="J91" s="2"/>
     </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A92" s="2"/>
       <c r="B92" s="2"/>
       <c r="C92" s="2"/>
@@ -5197,7 +5204,7 @@
       <c r="I92" s="2"/>
       <c r="J92" s="2"/>
     </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A93" s="2"/>
       <c r="B93" s="2"/>
       <c r="C93" s="2"/>
@@ -5209,7 +5216,7 @@
       <c r="I93" s="2"/>
       <c r="J93" s="2"/>
     </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A94" s="2"/>
       <c r="B94" s="2"/>
       <c r="C94" s="2"/>
@@ -5221,7 +5228,7 @@
       <c r="I94" s="2"/>
       <c r="J94" s="2"/>
     </row>
-    <row r="95" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A95" s="2"/>
       <c r="B95" s="2"/>
       <c r="C95" s="2"/>
@@ -5233,7 +5240,7 @@
       <c r="I95" s="2"/>
       <c r="J95" s="2"/>
     </row>
-    <row r="96" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A96" s="2"/>
       <c r="B96" s="2"/>
       <c r="C96" s="2"/>
@@ -5245,7 +5252,7 @@
       <c r="I96" s="2"/>
       <c r="J96" s="2"/>
     </row>
-    <row r="97" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A97" s="2"/>
       <c r="B97" s="2"/>
       <c r="C97" s="2"/>
@@ -5257,7 +5264,7 @@
       <c r="I97" s="2"/>
       <c r="J97" s="2"/>
     </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A98" s="2"/>
       <c r="B98" s="2"/>
       <c r="C98" s="2"/>
@@ -5269,7 +5276,7 @@
       <c r="I98" s="2"/>
       <c r="J98" s="2"/>
     </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A99" s="2"/>
       <c r="B99" s="2"/>
       <c r="C99" s="2"/>
@@ -5281,7 +5288,7 @@
       <c r="I99" s="2"/>
       <c r="J99" s="2"/>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A100" s="2"/>
       <c r="B100" s="2"/>
       <c r="C100" s="2"/>
@@ -5319,31 +5326,31 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:AA100"/>
-  <sheetFormatPr defaultColWidth="9.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.33203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="20.7109375" style="3" customWidth="1"/>
-    <col min="2" max="2" width="6.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="10" width="20.7109375" style="3" customWidth="1"/>
-    <col min="11" max="11" width="13.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="14.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="17.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="10.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="13.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.6640625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="6.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="10" width="20.6640625" style="3" customWidth="1"/>
+    <col min="11" max="11" width="13.5" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.5" style="3" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="14.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="17.1640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="10.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="13.6640625" style="2" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="12" style="2" customWidth="1"/>
-    <col min="22" max="22" width="9.28515625" style="2"/>
-    <col min="23" max="23" width="10.85546875" style="2" customWidth="1"/>
-    <col min="24" max="24" width="11.7109375" style="2" customWidth="1"/>
+    <col min="22" max="22" width="9.33203125" style="2"/>
+    <col min="23" max="23" width="10.83203125" style="2" customWidth="1"/>
+    <col min="24" max="24" width="11.6640625" style="2" customWidth="1"/>
     <col min="25" max="25" width="10" style="2" customWidth="1"/>
-    <col min="26" max="26" width="14.28515625" style="2" customWidth="1"/>
-    <col min="27" max="27" width="13.85546875" style="2" customWidth="1"/>
+    <col min="26" max="26" width="14.33203125" style="2" customWidth="1"/>
+    <col min="27" max="27" width="13.83203125" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" s="12" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:27" s="12" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>29</v>
       </c>
@@ -5426,7 +5433,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:27" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:27" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="4"/>
       <c r="C2" s="5"/>
       <c r="D2" s="5"/>
@@ -5450,7 +5457,7 @@
       <c r="Z2" s="11"/>
       <c r="AA2" s="11"/>
     </row>
-    <row r="3" spans="1:27" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:27" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="9"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -5475,7 +5482,7 @@
       <c r="Z3" s="11"/>
       <c r="AA3" s="11"/>
     </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -5496,7 +5503,7 @@
       <c r="R4" s="2"/>
       <c r="S4" s="2"/>
     </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -5517,7 +5524,7 @@
       <c r="R5" s="2"/>
       <c r="S5" s="2"/>
     </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -5538,7 +5545,7 @@
       <c r="R6" s="2"/>
       <c r="S6" s="2"/>
     </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -5559,7 +5566,7 @@
       <c r="R7" s="2"/>
       <c r="S7" s="2"/>
     </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -5580,7 +5587,7 @@
       <c r="R8" s="2"/>
       <c r="S8" s="2"/>
     </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -5601,7 +5608,7 @@
       <c r="R9" s="2"/>
       <c r="S9" s="2"/>
     </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -5622,7 +5629,7 @@
       <c r="R10" s="2"/>
       <c r="S10" s="2"/>
     </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -5643,7 +5650,7 @@
       <c r="R11" s="2"/>
       <c r="S11" s="2"/>
     </row>
-    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -5664,7 +5671,7 @@
       <c r="R12" s="2"/>
       <c r="S12" s="2"/>
     </row>
-    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -5685,7 +5692,7 @@
       <c r="R13" s="2"/>
       <c r="S13" s="2"/>
     </row>
-    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -5706,7 +5713,7 @@
       <c r="R14" s="2"/>
       <c r="S14" s="2"/>
     </row>
-    <row r="15" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -5727,7 +5734,7 @@
       <c r="R15" s="2"/>
       <c r="S15" s="2"/>
     </row>
-    <row r="16" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -5748,7 +5755,7 @@
       <c r="R16" s="2"/>
       <c r="S16" s="2"/>
     </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A17" s="2"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -5769,7 +5776,7 @@
       <c r="R17" s="2"/>
       <c r="S17" s="2"/>
     </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -5790,7 +5797,7 @@
       <c r="R18" s="2"/>
       <c r="S18" s="2"/>
     </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -5811,7 +5818,7 @@
       <c r="R19" s="2"/>
       <c r="S19" s="2"/>
     </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -5832,7 +5839,7 @@
       <c r="R20" s="2"/>
       <c r="S20" s="2"/>
     </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
@@ -5853,7 +5860,7 @@
       <c r="R21" s="2"/>
       <c r="S21" s="2"/>
     </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
@@ -5874,7 +5881,7 @@
       <c r="R22" s="2"/>
       <c r="S22" s="2"/>
     </row>
-    <row r="23" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A23" s="2"/>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
@@ -5895,7 +5902,7 @@
       <c r="R23" s="2"/>
       <c r="S23" s="2"/>
     </row>
-    <row r="24" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
@@ -5916,7 +5923,7 @@
       <c r="R24" s="2"/>
       <c r="S24" s="2"/>
     </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
@@ -5937,7 +5944,7 @@
       <c r="R25" s="2"/>
       <c r="S25" s="2"/>
     </row>
-    <row r="26" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
@@ -5958,7 +5965,7 @@
       <c r="R26" s="2"/>
       <c r="S26" s="2"/>
     </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
@@ -5979,7 +5986,7 @@
       <c r="R27" s="2"/>
       <c r="S27" s="2"/>
     </row>
-    <row r="28" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
@@ -6000,7 +6007,7 @@
       <c r="R28" s="2"/>
       <c r="S28" s="2"/>
     </row>
-    <row r="29" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
@@ -6021,7 +6028,7 @@
       <c r="R29" s="2"/>
       <c r="S29" s="2"/>
     </row>
-    <row r="30" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A30" s="2"/>
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
@@ -6042,7 +6049,7 @@
       <c r="R30" s="2"/>
       <c r="S30" s="2"/>
     </row>
-    <row r="31" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
@@ -6063,7 +6070,7 @@
       <c r="R31" s="2"/>
       <c r="S31" s="2"/>
     </row>
-    <row r="32" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
@@ -6084,7 +6091,7 @@
       <c r="R32" s="2"/>
       <c r="S32" s="2"/>
     </row>
-    <row r="33" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
@@ -6105,7 +6112,7 @@
       <c r="R33" s="2"/>
       <c r="S33" s="2"/>
     </row>
-    <row r="34" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
@@ -6126,7 +6133,7 @@
       <c r="R34" s="2"/>
       <c r="S34" s="2"/>
     </row>
-    <row r="35" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A35" s="2"/>
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
@@ -6147,7 +6154,7 @@
       <c r="R35" s="2"/>
       <c r="S35" s="2"/>
     </row>
-    <row r="36" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
@@ -6168,7 +6175,7 @@
       <c r="R36" s="2"/>
       <c r="S36" s="2"/>
     </row>
-    <row r="37" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
@@ -6189,7 +6196,7 @@
       <c r="R37" s="2"/>
       <c r="S37" s="2"/>
     </row>
-    <row r="38" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A38" s="2"/>
       <c r="B38" s="2"/>
       <c r="C38" s="2"/>
@@ -6210,7 +6217,7 @@
       <c r="R38" s="2"/>
       <c r="S38" s="2"/>
     </row>
-    <row r="39" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A39" s="2"/>
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
@@ -6231,7 +6238,7 @@
       <c r="R39" s="2"/>
       <c r="S39" s="2"/>
     </row>
-    <row r="40" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A40" s="2"/>
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
@@ -6252,7 +6259,7 @@
       <c r="R40" s="2"/>
       <c r="S40" s="2"/>
     </row>
-    <row r="41" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A41" s="2"/>
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
@@ -6273,7 +6280,7 @@
       <c r="R41" s="2"/>
       <c r="S41" s="2"/>
     </row>
-    <row r="42" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A42" s="2"/>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
@@ -6294,7 +6301,7 @@
       <c r="R42" s="2"/>
       <c r="S42" s="2"/>
     </row>
-    <row r="43" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A43" s="2"/>
       <c r="B43" s="2"/>
       <c r="C43" s="2"/>
@@ -6315,7 +6322,7 @@
       <c r="R43" s="2"/>
       <c r="S43" s="2"/>
     </row>
-    <row r="44" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A44" s="2"/>
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
@@ -6336,7 +6343,7 @@
       <c r="R44" s="2"/>
       <c r="S44" s="2"/>
     </row>
-    <row r="45" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A45" s="2"/>
       <c r="B45" s="2"/>
       <c r="C45" s="2"/>
@@ -6357,7 +6364,7 @@
       <c r="R45" s="2"/>
       <c r="S45" s="2"/>
     </row>
-    <row r="46" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A46" s="2"/>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
@@ -6378,7 +6385,7 @@
       <c r="R46" s="2"/>
       <c r="S46" s="2"/>
     </row>
-    <row r="47" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A47" s="2"/>
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
@@ -6399,7 +6406,7 @@
       <c r="R47" s="2"/>
       <c r="S47" s="2"/>
     </row>
-    <row r="48" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A48" s="2"/>
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
@@ -6420,7 +6427,7 @@
       <c r="R48" s="2"/>
       <c r="S48" s="2"/>
     </row>
-    <row r="49" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A49" s="2"/>
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
@@ -6441,7 +6448,7 @@
       <c r="R49" s="2"/>
       <c r="S49" s="2"/>
     </row>
-    <row r="50" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A50" s="2"/>
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
@@ -6462,7 +6469,7 @@
       <c r="R50" s="2"/>
       <c r="S50" s="2"/>
     </row>
-    <row r="51" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A51" s="2"/>
       <c r="B51" s="2"/>
       <c r="C51" s="2"/>
@@ -6483,7 +6490,7 @@
       <c r="R51" s="2"/>
       <c r="S51" s="2"/>
     </row>
-    <row r="52" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A52" s="2"/>
       <c r="B52" s="2"/>
       <c r="C52" s="2"/>
@@ -6504,7 +6511,7 @@
       <c r="R52" s="2"/>
       <c r="S52" s="2"/>
     </row>
-    <row r="53" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A53" s="2"/>
       <c r="B53" s="2"/>
       <c r="C53" s="2"/>
@@ -6525,7 +6532,7 @@
       <c r="R53" s="2"/>
       <c r="S53" s="2"/>
     </row>
-    <row r="54" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A54" s="2"/>
       <c r="B54" s="2"/>
       <c r="C54" s="2"/>
@@ -6546,7 +6553,7 @@
       <c r="R54" s="2"/>
       <c r="S54" s="2"/>
     </row>
-    <row r="55" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A55" s="2"/>
       <c r="B55" s="2"/>
       <c r="C55" s="2"/>
@@ -6567,7 +6574,7 @@
       <c r="R55" s="2"/>
       <c r="S55" s="2"/>
     </row>
-    <row r="56" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A56" s="2"/>
       <c r="B56" s="2"/>
       <c r="C56" s="2"/>
@@ -6588,7 +6595,7 @@
       <c r="R56" s="2"/>
       <c r="S56" s="2"/>
     </row>
-    <row r="57" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A57" s="2"/>
       <c r="B57" s="2"/>
       <c r="C57" s="2"/>
@@ -6609,7 +6616,7 @@
       <c r="R57" s="2"/>
       <c r="S57" s="2"/>
     </row>
-    <row r="58" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A58" s="2"/>
       <c r="B58" s="2"/>
       <c r="C58" s="2"/>
@@ -6630,7 +6637,7 @@
       <c r="R58" s="2"/>
       <c r="S58" s="2"/>
     </row>
-    <row r="59" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A59" s="2"/>
       <c r="B59" s="2"/>
       <c r="C59" s="2"/>
@@ -6651,7 +6658,7 @@
       <c r="R59" s="2"/>
       <c r="S59" s="2"/>
     </row>
-    <row r="60" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A60" s="2"/>
       <c r="B60" s="2"/>
       <c r="C60" s="2"/>
@@ -6672,7 +6679,7 @@
       <c r="R60" s="2"/>
       <c r="S60" s="2"/>
     </row>
-    <row r="61" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A61" s="2"/>
       <c r="B61" s="2"/>
       <c r="C61" s="2"/>
@@ -6693,7 +6700,7 @@
       <c r="R61" s="2"/>
       <c r="S61" s="2"/>
     </row>
-    <row r="62" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A62" s="2"/>
       <c r="B62" s="2"/>
       <c r="C62" s="2"/>
@@ -6714,7 +6721,7 @@
       <c r="R62" s="2"/>
       <c r="S62" s="2"/>
     </row>
-    <row r="63" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A63" s="2"/>
       <c r="B63" s="2"/>
       <c r="C63" s="2"/>
@@ -6735,7 +6742,7 @@
       <c r="R63" s="2"/>
       <c r="S63" s="2"/>
     </row>
-    <row r="64" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A64" s="2"/>
       <c r="B64" s="2"/>
       <c r="C64" s="2"/>
@@ -6756,7 +6763,7 @@
       <c r="R64" s="2"/>
       <c r="S64" s="2"/>
     </row>
-    <row r="65" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A65" s="2"/>
       <c r="B65" s="2"/>
       <c r="C65" s="2"/>
@@ -6777,7 +6784,7 @@
       <c r="R65" s="2"/>
       <c r="S65" s="2"/>
     </row>
-    <row r="66" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A66" s="2"/>
       <c r="B66" s="2"/>
       <c r="C66" s="2"/>
@@ -6798,7 +6805,7 @@
       <c r="R66" s="2"/>
       <c r="S66" s="2"/>
     </row>
-    <row r="67" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A67" s="2"/>
       <c r="B67" s="2"/>
       <c r="C67" s="2"/>
@@ -6819,7 +6826,7 @@
       <c r="R67" s="2"/>
       <c r="S67" s="2"/>
     </row>
-    <row r="68" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A68" s="2"/>
       <c r="B68" s="2"/>
       <c r="C68" s="2"/>
@@ -6840,7 +6847,7 @@
       <c r="R68" s="2"/>
       <c r="S68" s="2"/>
     </row>
-    <row r="69" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A69" s="2"/>
       <c r="B69" s="2"/>
       <c r="C69" s="2"/>
@@ -6861,7 +6868,7 @@
       <c r="R69" s="2"/>
       <c r="S69" s="2"/>
     </row>
-    <row r="70" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A70" s="2"/>
       <c r="B70" s="2"/>
       <c r="C70" s="2"/>
@@ -6882,7 +6889,7 @@
       <c r="R70" s="2"/>
       <c r="S70" s="2"/>
     </row>
-    <row r="71" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A71" s="2"/>
       <c r="B71" s="2"/>
       <c r="C71" s="2"/>
@@ -6903,7 +6910,7 @@
       <c r="R71" s="2"/>
       <c r="S71" s="2"/>
     </row>
-    <row r="72" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A72" s="2"/>
       <c r="B72" s="2"/>
       <c r="C72" s="2"/>
@@ -6924,7 +6931,7 @@
       <c r="R72" s="2"/>
       <c r="S72" s="2"/>
     </row>
-    <row r="73" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A73" s="2"/>
       <c r="B73" s="2"/>
       <c r="C73" s="2"/>
@@ -6945,7 +6952,7 @@
       <c r="R73" s="2"/>
       <c r="S73" s="2"/>
     </row>
-    <row r="74" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A74" s="2"/>
       <c r="B74" s="2"/>
       <c r="C74" s="2"/>
@@ -6966,7 +6973,7 @@
       <c r="R74" s="2"/>
       <c r="S74" s="2"/>
     </row>
-    <row r="75" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A75" s="2"/>
       <c r="B75" s="2"/>
       <c r="C75" s="2"/>
@@ -6987,7 +6994,7 @@
       <c r="R75" s="2"/>
       <c r="S75" s="2"/>
     </row>
-    <row r="76" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A76" s="2"/>
       <c r="B76" s="2"/>
       <c r="C76" s="2"/>
@@ -7008,7 +7015,7 @@
       <c r="R76" s="2"/>
       <c r="S76" s="2"/>
     </row>
-    <row r="77" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A77" s="2"/>
       <c r="B77" s="2"/>
       <c r="C77" s="2"/>
@@ -7029,7 +7036,7 @@
       <c r="R77" s="2"/>
       <c r="S77" s="2"/>
     </row>
-    <row r="78" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A78" s="2"/>
       <c r="B78" s="2"/>
       <c r="C78" s="2"/>
@@ -7050,7 +7057,7 @@
       <c r="R78" s="2"/>
       <c r="S78" s="2"/>
     </row>
-    <row r="79" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A79" s="2"/>
       <c r="B79" s="2"/>
       <c r="C79" s="2"/>
@@ -7071,7 +7078,7 @@
       <c r="R79" s="2"/>
       <c r="S79" s="2"/>
     </row>
-    <row r="80" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A80" s="2"/>
       <c r="B80" s="2"/>
       <c r="C80" s="2"/>
@@ -7092,7 +7099,7 @@
       <c r="R80" s="2"/>
       <c r="S80" s="2"/>
     </row>
-    <row r="81" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A81" s="2"/>
       <c r="B81" s="2"/>
       <c r="C81" s="2"/>
@@ -7113,7 +7120,7 @@
       <c r="R81" s="2"/>
       <c r="S81" s="2"/>
     </row>
-    <row r="82" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A82" s="2"/>
       <c r="B82" s="2"/>
       <c r="C82" s="2"/>
@@ -7134,7 +7141,7 @@
       <c r="R82" s="2"/>
       <c r="S82" s="2"/>
     </row>
-    <row r="83" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A83" s="2"/>
       <c r="B83" s="2"/>
       <c r="C83" s="2"/>
@@ -7155,7 +7162,7 @@
       <c r="R83" s="2"/>
       <c r="S83" s="2"/>
     </row>
-    <row r="84" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A84" s="2"/>
       <c r="B84" s="2"/>
       <c r="C84" s="2"/>
@@ -7176,7 +7183,7 @@
       <c r="R84" s="2"/>
       <c r="S84" s="2"/>
     </row>
-    <row r="85" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A85" s="2"/>
       <c r="B85" s="2"/>
       <c r="C85" s="2"/>
@@ -7197,7 +7204,7 @@
       <c r="R85" s="2"/>
       <c r="S85" s="2"/>
     </row>
-    <row r="86" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A86" s="2"/>
       <c r="B86" s="2"/>
       <c r="C86" s="2"/>
@@ -7218,7 +7225,7 @@
       <c r="R86" s="2"/>
       <c r="S86" s="2"/>
     </row>
-    <row r="87" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A87" s="2"/>
       <c r="B87" s="2"/>
       <c r="C87" s="2"/>
@@ -7239,7 +7246,7 @@
       <c r="R87" s="2"/>
       <c r="S87" s="2"/>
     </row>
-    <row r="88" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A88" s="2"/>
       <c r="B88" s="2"/>
       <c r="C88" s="2"/>
@@ -7260,7 +7267,7 @@
       <c r="R88" s="2"/>
       <c r="S88" s="2"/>
     </row>
-    <row r="89" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A89" s="2"/>
       <c r="B89" s="2"/>
       <c r="C89" s="2"/>
@@ -7281,7 +7288,7 @@
       <c r="R89" s="2"/>
       <c r="S89" s="2"/>
     </row>
-    <row r="90" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A90" s="2"/>
       <c r="B90" s="2"/>
       <c r="C90" s="2"/>
@@ -7302,7 +7309,7 @@
       <c r="R90" s="2"/>
       <c r="S90" s="2"/>
     </row>
-    <row r="91" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A91" s="2"/>
       <c r="B91" s="2"/>
       <c r="C91" s="2"/>
@@ -7323,7 +7330,7 @@
       <c r="R91" s="2"/>
       <c r="S91" s="2"/>
     </row>
-    <row r="92" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A92" s="2"/>
       <c r="B92" s="2"/>
       <c r="C92" s="2"/>
@@ -7344,7 +7351,7 @@
       <c r="R92" s="2"/>
       <c r="S92" s="2"/>
     </row>
-    <row r="93" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A93" s="2"/>
       <c r="B93" s="2"/>
       <c r="C93" s="2"/>
@@ -7365,7 +7372,7 @@
       <c r="R93" s="2"/>
       <c r="S93" s="2"/>
     </row>
-    <row r="94" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A94" s="2"/>
       <c r="B94" s="2"/>
       <c r="C94" s="2"/>
@@ -7386,7 +7393,7 @@
       <c r="R94" s="2"/>
       <c r="S94" s="2"/>
     </row>
-    <row r="95" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A95" s="2"/>
       <c r="B95" s="2"/>
       <c r="C95" s="2"/>
@@ -7407,7 +7414,7 @@
       <c r="R95" s="2"/>
       <c r="S95" s="2"/>
     </row>
-    <row r="96" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A96" s="2"/>
       <c r="B96" s="2"/>
       <c r="C96" s="2"/>
@@ -7428,7 +7435,7 @@
       <c r="R96" s="2"/>
       <c r="S96" s="2"/>
     </row>
-    <row r="97" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A97" s="2"/>
       <c r="B97" s="2"/>
       <c r="C97" s="2"/>
@@ -7449,7 +7456,7 @@
       <c r="R97" s="2"/>
       <c r="S97" s="2"/>
     </row>
-    <row r="98" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A98" s="2"/>
       <c r="B98" s="2"/>
       <c r="C98" s="2"/>
@@ -7470,7 +7477,7 @@
       <c r="R98" s="2"/>
       <c r="S98" s="2"/>
     </row>
-    <row r="99" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A99" s="2"/>
       <c r="B99" s="2"/>
       <c r="C99" s="2"/>
@@ -7491,7 +7498,7 @@
       <c r="R99" s="2"/>
       <c r="S99" s="2"/>
     </row>
-    <row r="100" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A100" s="2"/>
       <c r="B100" s="2"/>
       <c r="C100" s="2"/>
@@ -7540,14 +7547,14 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:F100"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="20.7109375" style="3" customWidth="1"/>
-    <col min="2" max="2" width="6.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="6" width="20.7109375" style="3" customWidth="1"/>
+    <col min="1" max="1" width="20.6640625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="6.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="6" width="20.6640625" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>29</v>
       </c>
@@ -7567,14 +7574,14 @@
         <v>64</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="4"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="9"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -7582,7 +7589,7 @@
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -7590,7 +7597,7 @@
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -7598,7 +7605,7 @@
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -7606,7 +7613,7 @@
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -7614,7 +7621,7 @@
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -7622,7 +7629,7 @@
       <c r="E8" s="2"/>
       <c r="F8" s="2"/>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -7630,7 +7637,7 @@
       <c r="E9" s="2"/>
       <c r="F9" s="2"/>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -7638,7 +7645,7 @@
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -7646,7 +7653,7 @@
       <c r="E11" s="2"/>
       <c r="F11" s="2"/>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -7654,7 +7661,7 @@
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -7662,7 +7669,7 @@
       <c r="E13" s="2"/>
       <c r="F13" s="2"/>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -7670,7 +7677,7 @@
       <c r="E14" s="2"/>
       <c r="F14" s="2"/>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -7678,7 +7685,7 @@
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -7686,7 +7693,7 @@
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="2"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -7694,7 +7701,7 @@
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -7702,7 +7709,7 @@
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -7710,7 +7717,7 @@
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -7718,7 +7725,7 @@
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
@@ -7726,7 +7733,7 @@
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
@@ -7734,7 +7741,7 @@
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" s="2"/>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
@@ -7742,7 +7749,7 @@
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
@@ -7750,7 +7757,7 @@
       <c r="E24" s="2"/>
       <c r="F24" s="2"/>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
@@ -7758,7 +7765,7 @@
       <c r="E25" s="2"/>
       <c r="F25" s="2"/>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
@@ -7766,7 +7773,7 @@
       <c r="E26" s="2"/>
       <c r="F26" s="2"/>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
@@ -7774,7 +7781,7 @@
       <c r="E27" s="2"/>
       <c r="F27" s="2"/>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
@@ -7782,7 +7789,7 @@
       <c r="E28" s="2"/>
       <c r="F28" s="2"/>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
@@ -7790,7 +7797,7 @@
       <c r="E29" s="2"/>
       <c r="F29" s="2"/>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" s="2"/>
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
@@ -7798,7 +7805,7 @@
       <c r="E30" s="2"/>
       <c r="F30" s="2"/>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
@@ -7806,7 +7813,7 @@
       <c r="E31" s="2"/>
       <c r="F31" s="2"/>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
@@ -7814,7 +7821,7 @@
       <c r="E32" s="2"/>
       <c r="F32" s="2"/>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
@@ -7822,7 +7829,7 @@
       <c r="E33" s="2"/>
       <c r="F33" s="2"/>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
@@ -7830,7 +7837,7 @@
       <c r="E34" s="2"/>
       <c r="F34" s="2"/>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35" s="2"/>
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
@@ -7838,7 +7845,7 @@
       <c r="E35" s="2"/>
       <c r="F35" s="2"/>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
@@ -7846,7 +7853,7 @@
       <c r="E36" s="2"/>
       <c r="F36" s="2"/>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
@@ -7854,7 +7861,7 @@
       <c r="E37" s="2"/>
       <c r="F37" s="2"/>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38" s="2"/>
       <c r="B38" s="2"/>
       <c r="C38" s="2"/>
@@ -7862,7 +7869,7 @@
       <c r="E38" s="2"/>
       <c r="F38" s="2"/>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A39" s="2"/>
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
@@ -7870,7 +7877,7 @@
       <c r="E39" s="2"/>
       <c r="F39" s="2"/>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A40" s="2"/>
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
@@ -7878,7 +7885,7 @@
       <c r="E40" s="2"/>
       <c r="F40" s="2"/>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41" s="2"/>
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
@@ -7886,7 +7893,7 @@
       <c r="E41" s="2"/>
       <c r="F41" s="2"/>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42" s="2"/>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
@@ -7894,7 +7901,7 @@
       <c r="E42" s="2"/>
       <c r="F42" s="2"/>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43" s="2"/>
       <c r="B43" s="2"/>
       <c r="C43" s="2"/>
@@ -7902,7 +7909,7 @@
       <c r="E43" s="2"/>
       <c r="F43" s="2"/>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A44" s="2"/>
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
@@ -7910,7 +7917,7 @@
       <c r="E44" s="2"/>
       <c r="F44" s="2"/>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45" s="2"/>
       <c r="B45" s="2"/>
       <c r="C45" s="2"/>
@@ -7918,7 +7925,7 @@
       <c r="E45" s="2"/>
       <c r="F45" s="2"/>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A46" s="2"/>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
@@ -7926,7 +7933,7 @@
       <c r="E46" s="2"/>
       <c r="F46" s="2"/>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A47" s="2"/>
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
@@ -7934,7 +7941,7 @@
       <c r="E47" s="2"/>
       <c r="F47" s="2"/>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A48" s="2"/>
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
@@ -7942,7 +7949,7 @@
       <c r="E48" s="2"/>
       <c r="F48" s="2"/>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A49" s="2"/>
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
@@ -7950,7 +7957,7 @@
       <c r="E49" s="2"/>
       <c r="F49" s="2"/>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A50" s="2"/>
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
@@ -7958,7 +7965,7 @@
       <c r="E50" s="2"/>
       <c r="F50" s="2"/>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A51" s="2"/>
       <c r="B51" s="2"/>
       <c r="C51" s="2"/>
@@ -7966,7 +7973,7 @@
       <c r="E51" s="2"/>
       <c r="F51" s="2"/>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A52" s="2"/>
       <c r="B52" s="2"/>
       <c r="C52" s="2"/>
@@ -7974,7 +7981,7 @@
       <c r="E52" s="2"/>
       <c r="F52" s="2"/>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A53" s="2"/>
       <c r="B53" s="2"/>
       <c r="C53" s="2"/>
@@ -7982,7 +7989,7 @@
       <c r="E53" s="2"/>
       <c r="F53" s="2"/>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A54" s="2"/>
       <c r="B54" s="2"/>
       <c r="C54" s="2"/>
@@ -7990,7 +7997,7 @@
       <c r="E54" s="2"/>
       <c r="F54" s="2"/>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A55" s="2"/>
       <c r="B55" s="2"/>
       <c r="C55" s="2"/>
@@ -7998,7 +8005,7 @@
       <c r="E55" s="2"/>
       <c r="F55" s="2"/>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A56" s="2"/>
       <c r="B56" s="2"/>
       <c r="C56" s="2"/>
@@ -8006,7 +8013,7 @@
       <c r="E56" s="2"/>
       <c r="F56" s="2"/>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A57" s="2"/>
       <c r="B57" s="2"/>
       <c r="C57" s="2"/>
@@ -8014,7 +8021,7 @@
       <c r="E57" s="2"/>
       <c r="F57" s="2"/>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A58" s="2"/>
       <c r="B58" s="2"/>
       <c r="C58" s="2"/>
@@ -8022,7 +8029,7 @@
       <c r="E58" s="2"/>
       <c r="F58" s="2"/>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A59" s="2"/>
       <c r="B59" s="2"/>
       <c r="C59" s="2"/>
@@ -8030,7 +8037,7 @@
       <c r="E59" s="2"/>
       <c r="F59" s="2"/>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A60" s="2"/>
       <c r="B60" s="2"/>
       <c r="C60" s="2"/>
@@ -8038,7 +8045,7 @@
       <c r="E60" s="2"/>
       <c r="F60" s="2"/>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A61" s="2"/>
       <c r="B61" s="2"/>
       <c r="C61" s="2"/>
@@ -8046,7 +8053,7 @@
       <c r="E61" s="2"/>
       <c r="F61" s="2"/>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A62" s="2"/>
       <c r="B62" s="2"/>
       <c r="C62" s="2"/>
@@ -8054,7 +8061,7 @@
       <c r="E62" s="2"/>
       <c r="F62" s="2"/>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A63" s="2"/>
       <c r="B63" s="2"/>
       <c r="C63" s="2"/>
@@ -8062,7 +8069,7 @@
       <c r="E63" s="2"/>
       <c r="F63" s="2"/>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A64" s="2"/>
       <c r="B64" s="2"/>
       <c r="C64" s="2"/>
@@ -8070,7 +8077,7 @@
       <c r="E64" s="2"/>
       <c r="F64" s="2"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A65" s="2"/>
       <c r="B65" s="2"/>
       <c r="C65" s="2"/>
@@ -8078,7 +8085,7 @@
       <c r="E65" s="2"/>
       <c r="F65" s="2"/>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A66" s="2"/>
       <c r="B66" s="2"/>
       <c r="C66" s="2"/>
@@ -8086,7 +8093,7 @@
       <c r="E66" s="2"/>
       <c r="F66" s="2"/>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A67" s="2"/>
       <c r="B67" s="2"/>
       <c r="C67" s="2"/>
@@ -8094,7 +8101,7 @@
       <c r="E67" s="2"/>
       <c r="F67" s="2"/>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A68" s="2"/>
       <c r="B68" s="2"/>
       <c r="C68" s="2"/>
@@ -8102,7 +8109,7 @@
       <c r="E68" s="2"/>
       <c r="F68" s="2"/>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A69" s="2"/>
       <c r="B69" s="2"/>
       <c r="C69" s="2"/>
@@ -8110,7 +8117,7 @@
       <c r="E69" s="2"/>
       <c r="F69" s="2"/>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A70" s="2"/>
       <c r="B70" s="2"/>
       <c r="C70" s="2"/>
@@ -8118,7 +8125,7 @@
       <c r="E70" s="2"/>
       <c r="F70" s="2"/>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A71" s="2"/>
       <c r="B71" s="2"/>
       <c r="C71" s="2"/>
@@ -8126,7 +8133,7 @@
       <c r="E71" s="2"/>
       <c r="F71" s="2"/>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A72" s="2"/>
       <c r="B72" s="2"/>
       <c r="C72" s="2"/>
@@ -8134,7 +8141,7 @@
       <c r="E72" s="2"/>
       <c r="F72" s="2"/>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A73" s="2"/>
       <c r="B73" s="2"/>
       <c r="C73" s="2"/>
@@ -8142,7 +8149,7 @@
       <c r="E73" s="2"/>
       <c r="F73" s="2"/>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A74" s="2"/>
       <c r="B74" s="2"/>
       <c r="C74" s="2"/>
@@ -8150,7 +8157,7 @@
       <c r="E74" s="2"/>
       <c r="F74" s="2"/>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A75" s="2"/>
       <c r="B75" s="2"/>
       <c r="C75" s="2"/>
@@ -8158,7 +8165,7 @@
       <c r="E75" s="2"/>
       <c r="F75" s="2"/>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A76" s="2"/>
       <c r="B76" s="2"/>
       <c r="C76" s="2"/>
@@ -8166,7 +8173,7 @@
       <c r="E76" s="2"/>
       <c r="F76" s="2"/>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A77" s="2"/>
       <c r="B77" s="2"/>
       <c r="C77" s="2"/>
@@ -8174,7 +8181,7 @@
       <c r="E77" s="2"/>
       <c r="F77" s="2"/>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A78" s="2"/>
       <c r="B78" s="2"/>
       <c r="C78" s="2"/>
@@ -8182,7 +8189,7 @@
       <c r="E78" s="2"/>
       <c r="F78" s="2"/>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A79" s="2"/>
       <c r="B79" s="2"/>
       <c r="C79" s="2"/>
@@ -8190,7 +8197,7 @@
       <c r="E79" s="2"/>
       <c r="F79" s="2"/>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A80" s="2"/>
       <c r="B80" s="2"/>
       <c r="C80" s="2"/>
@@ -8198,7 +8205,7 @@
       <c r="E80" s="2"/>
       <c r="F80" s="2"/>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A81" s="2"/>
       <c r="B81" s="2"/>
       <c r="C81" s="2"/>
@@ -8206,7 +8213,7 @@
       <c r="E81" s="2"/>
       <c r="F81" s="2"/>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A82" s="2"/>
       <c r="B82" s="2"/>
       <c r="C82" s="2"/>
@@ -8214,7 +8221,7 @@
       <c r="E82" s="2"/>
       <c r="F82" s="2"/>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A83" s="2"/>
       <c r="B83" s="2"/>
       <c r="C83" s="2"/>
@@ -8222,7 +8229,7 @@
       <c r="E83" s="2"/>
       <c r="F83" s="2"/>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A84" s="2"/>
       <c r="B84" s="2"/>
       <c r="C84" s="2"/>
@@ -8230,7 +8237,7 @@
       <c r="E84" s="2"/>
       <c r="F84" s="2"/>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A85" s="2"/>
       <c r="B85" s="2"/>
       <c r="C85" s="2"/>
@@ -8238,7 +8245,7 @@
       <c r="E85" s="2"/>
       <c r="F85" s="2"/>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A86" s="2"/>
       <c r="B86" s="2"/>
       <c r="C86" s="2"/>
@@ -8246,7 +8253,7 @@
       <c r="E86" s="2"/>
       <c r="F86" s="2"/>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A87" s="2"/>
       <c r="B87" s="2"/>
       <c r="C87" s="2"/>
@@ -8254,7 +8261,7 @@
       <c r="E87" s="2"/>
       <c r="F87" s="2"/>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A88" s="2"/>
       <c r="B88" s="2"/>
       <c r="C88" s="2"/>
@@ -8262,7 +8269,7 @@
       <c r="E88" s="2"/>
       <c r="F88" s="2"/>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A89" s="2"/>
       <c r="B89" s="2"/>
       <c r="C89" s="2"/>
@@ -8270,7 +8277,7 @@
       <c r="E89" s="2"/>
       <c r="F89" s="2"/>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A90" s="2"/>
       <c r="B90" s="2"/>
       <c r="C90" s="2"/>
@@ -8278,7 +8285,7 @@
       <c r="E90" s="2"/>
       <c r="F90" s="2"/>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A91" s="2"/>
       <c r="B91" s="2"/>
       <c r="C91" s="2"/>
@@ -8286,7 +8293,7 @@
       <c r="E91" s="2"/>
       <c r="F91" s="2"/>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A92" s="2"/>
       <c r="B92" s="2"/>
       <c r="C92" s="2"/>
@@ -8294,7 +8301,7 @@
       <c r="E92" s="2"/>
       <c r="F92" s="2"/>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A93" s="2"/>
       <c r="B93" s="2"/>
       <c r="C93" s="2"/>
@@ -8302,7 +8309,7 @@
       <c r="E93" s="2"/>
       <c r="F93" s="2"/>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A94" s="2"/>
       <c r="B94" s="2"/>
       <c r="C94" s="2"/>
@@ -8310,7 +8317,7 @@
       <c r="E94" s="2"/>
       <c r="F94" s="2"/>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A95" s="2"/>
       <c r="B95" s="2"/>
       <c r="C95" s="2"/>
@@ -8318,7 +8325,7 @@
       <c r="E95" s="2"/>
       <c r="F95" s="2"/>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A96" s="2"/>
       <c r="B96" s="2"/>
       <c r="C96" s="2"/>
@@ -8326,7 +8333,7 @@
       <c r="E96" s="2"/>
       <c r="F96" s="2"/>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A97" s="2"/>
       <c r="B97" s="2"/>
       <c r="C97" s="2"/>
@@ -8334,7 +8341,7 @@
       <c r="E97" s="2"/>
       <c r="F97" s="2"/>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A98" s="2"/>
       <c r="B98" s="2"/>
       <c r="C98" s="2"/>
@@ -8342,7 +8349,7 @@
       <c r="E98" s="2"/>
       <c r="F98" s="2"/>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A99" s="2"/>
       <c r="B99" s="2"/>
       <c r="C99" s="2"/>
@@ -8350,7 +8357,7 @@
       <c r="E99" s="2"/>
       <c r="F99" s="2"/>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A100" s="2"/>
       <c r="B100" s="2"/>
       <c r="C100" s="2"/>

</xml_diff>